<commit_message>
Actualizadas testscases app-admin, y web
</commit_message>
<xml_diff>
--- a/App/TestCases_App/User_admin.xlsx
+++ b/App/TestCases_App/User_admin.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nerea QA\PycharmProjects\KOVAI\App\TestCases_App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DC53DEE-0F03-4126-A0D9-5A4BF7727F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20B6F5B4-72CB-4008-BFC2-519977461EC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="660">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="663">
   <si>
     <t>Num</t>
   </si>
@@ -604,9 +604,6 @@
   </si>
   <si>
     <t>No hace nada, se queda cargando, añadir funcionalidad</t>
-  </si>
-  <si>
-    <t>Aparece un mensaje de que "seleccione una serie de facturación" que no viene por ningún sitio: FAC002.jpg</t>
   </si>
   <si>
     <t>Aparece un mensaje de que "seleccione una serie de facturación" que no viene por ningún sitio FAC002.jpg</t>
@@ -2210,6 +2207,19 @@
 Al desplegar el teclado, se tapa la funcionalidad: MEN003.jpg
 Parece q me guarda el menú pero cuando voy a consultarlo, ha desaparecido.
 Se produce un error al guardar el menú: MEN005.jpg,MEN006.jpg</t>
+  </si>
+  <si>
+    <t>Al añadir modificadores, no se está teniendo en cuenta en la suma: PED001.jpg</t>
+  </si>
+  <si>
+    <t>Aparece un mensaje de que "seleccione una serie de facturación" que no viene por ningún sitio: FAC002.jpg
+En el restaurante Gran Via, me ha permitido generar factura, pero hay errores: FAC005.jpg y FAC006.jpg</t>
+  </si>
+  <si>
+    <t>1.The invoicing is created</t>
+  </si>
+  <si>
+    <t>1.The invoicing is not created</t>
   </si>
 </sst>
 </file>
@@ -2727,10 +2737,10 @@
         <v>36</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>579</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>580</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -2738,7 +2748,7 @@
         <v>8</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="4" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -2749,7 +2759,7 @@
         <v>37</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>9</v>
@@ -2760,7 +2770,7 @@
         <v>8</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="5" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -2771,7 +2781,7 @@
         <v>38</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>10</v>
@@ -2793,7 +2803,7 @@
         <v>39</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>12</v>
@@ -2815,7 +2825,7 @@
         <v>40</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>15</v>
@@ -2835,10 +2845,10 @@
         <v>41</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>587</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>588</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -2855,7 +2865,7 @@
         <v>42</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>13</v>
@@ -2863,9 +2873,11 @@
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H9" s="3"/>
+        <v>8</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>659</v>
+      </c>
     </row>
     <row r="10" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
@@ -2875,7 +2887,7 @@
         <v>43</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>14</v>
@@ -2895,7 +2907,7 @@
         <v>44</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>17</v>
@@ -2917,7 +2929,7 @@
         <v>45</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>22</v>
@@ -2941,7 +2953,7 @@
         <v>46</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>25</v>
@@ -2965,7 +2977,7 @@
         <v>47</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>26</v>
@@ -2989,7 +3001,7 @@
         <v>48</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>29</v>
@@ -3013,7 +3025,7 @@
         <v>49</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>90</v>
@@ -3037,7 +3049,7 @@
         <v>64</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>91</v>
@@ -3059,7 +3071,7 @@
         <v>65</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>94</v>
@@ -3081,7 +3093,7 @@
         <v>66</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>95</v>
@@ -3103,7 +3115,7 @@
         <v>67</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>98</v>
@@ -3197,7 +3209,7 @@
         <v>71</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>129</v>
@@ -3223,13 +3235,13 @@
         <v>83</v>
       </c>
       <c r="C25" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>589</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>590</v>
-      </c>
       <c r="E25" s="1" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="F25" s="1"/>
       <c r="G25" s="2" t="s">
@@ -3256,7 +3268,7 @@
         <v>20</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="27" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -3309,17 +3321,17 @@
         <v>137</v>
       </c>
       <c r="D29" s="1" t="s">
+        <v>653</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>654</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>655</v>
       </c>
       <c r="F29" s="1"/>
       <c r="G29" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="30" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -3341,7 +3353,7 @@
         <v>8</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="31" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3361,7 +3373,7 @@
         <v>20</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="32" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -3377,13 +3389,17 @@
       <c r="D32" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
+      <c r="E32" s="1" t="s">
+        <v>661</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>662</v>
+      </c>
       <c r="G32" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>167</v>
+        <v>660</v>
       </c>
     </row>
     <row r="33" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -3405,7 +3421,7 @@
         <v>20</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="34" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -3475,7 +3491,7 @@
         <v>20</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="37" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3541,7 +3557,7 @@
         <v>8</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="40" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3549,10 +3565,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>164</v>
@@ -3563,7 +3579,7 @@
         <v>8</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="41" spans="1:8" s="6" customFormat="1" ht="105" x14ac:dyDescent="0.25">
@@ -3571,23 +3587,23 @@
         <v>39</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C41" s="1" t="s">
+        <v>647</v>
+      </c>
+      <c r="D41" s="1" t="s">
         <v>648</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="E41" s="1" t="s">
         <v>649</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>650</v>
       </c>
       <c r="F41" s="1"/>
       <c r="G41" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="42" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -3595,13 +3611,13 @@
         <v>39</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C42" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>651</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>652</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>128</v>
@@ -3619,13 +3635,13 @@
         <v>40</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>
@@ -3633,7 +3649,7 @@
         <v>8</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="44" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3641,13 +3657,13 @@
         <v>41</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="E44" s="1"/>
       <c r="F44" s="1"/>
@@ -3655,7 +3671,7 @@
         <v>8</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="45" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -3663,13 +3679,13 @@
         <v>42</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C45" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>447</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>448</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -3677,7 +3693,7 @@
         <v>19</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="46" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -3685,19 +3701,19 @@
         <v>43</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="D46" s="1" t="s">
+        <v>612</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>613</v>
       </c>
-      <c r="E46" s="1" t="s">
-        <v>614</v>
-      </c>
       <c r="F46" s="1" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>19</v>
@@ -3709,19 +3725,19 @@
         <v>44</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="D47" s="1" t="s">
+        <v>614</v>
+      </c>
+      <c r="E47" s="1" t="s">
         <v>615</v>
       </c>
-      <c r="E47" s="1" t="s">
-        <v>616</v>
-      </c>
       <c r="F47" s="1" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="G47" s="2" t="s">
         <v>19</v>
@@ -3736,20 +3752,20 @@
         <v>111</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="F48" s="1"/>
       <c r="G48" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="49" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3760,10 +3776,10 @@
         <v>112</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>128</v>
@@ -3783,20 +3799,20 @@
         <v>113</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="D50" s="1" t="s">
+        <v>617</v>
+      </c>
+      <c r="E50" s="1" t="s">
         <v>618</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>619</v>
       </c>
       <c r="F50" s="1"/>
       <c r="G50" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="51" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -3807,10 +3823,10 @@
         <v>114</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>128</v>
@@ -3829,20 +3845,20 @@
         <v>115</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D52" s="1" t="s">
+        <v>645</v>
+      </c>
+      <c r="E52" s="1" t="s">
         <v>646</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>647</v>
       </c>
       <c r="F52" s="1"/>
       <c r="G52" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="53" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -3853,20 +3869,20 @@
         <v>116</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="F53" s="1"/>
       <c r="G53" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="54" spans="1:8" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -3877,20 +3893,20 @@
         <v>117</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="F54" s="1"/>
       <c r="G54" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="55" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3901,10 +3917,10 @@
         <v>118</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>128</v>
@@ -3922,23 +3938,23 @@
         <v>53</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="F56" s="1"/>
       <c r="G56" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="57" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3949,10 +3965,10 @@
         <v>119</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>128</v>
@@ -3973,16 +3989,16 @@
         <v>120</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="D58" s="1" t="s">
+        <v>641</v>
+      </c>
+      <c r="E58" s="1" t="s">
         <v>642</v>
       </c>
-      <c r="E58" s="1" t="s">
-        <v>643</v>
-      </c>
       <c r="F58" s="1" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="G58" s="2" t="s">
         <v>19</v>
@@ -3994,13 +4010,13 @@
         <v>56</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>128</v>
@@ -4021,16 +4037,16 @@
         <v>121</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="G60" s="2" t="s">
         <v>19</v>
@@ -4044,7 +4060,7 @@
         <v>122</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>139</v>
@@ -4064,16 +4080,16 @@
         <v>123</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="D62" s="1" t="s">
+        <v>604</v>
+      </c>
+      <c r="E62" s="1" t="s">
         <v>605</v>
       </c>
-      <c r="E62" s="1" t="s">
-        <v>606</v>
-      </c>
       <c r="F62" s="1" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="G62" s="2" t="s">
         <v>19</v>
@@ -4088,10 +4104,10 @@
         <v>124</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>128</v>
@@ -4112,16 +4128,16 @@
         <v>125</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>19</v>
@@ -4136,10 +4152,10 @@
         <v>126</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>128</v>
@@ -4160,16 +4176,16 @@
         <v>127</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="D66" s="1" t="s">
+        <v>610</v>
+      </c>
+      <c r="E66" s="1" t="s">
         <v>611</v>
       </c>
-      <c r="E66" s="1" t="s">
-        <v>612</v>
-      </c>
       <c r="F66" s="1" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="G66" s="2" t="s">
         <v>19</v>
@@ -4181,13 +4197,13 @@
         <v>64</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>128</v>
@@ -4205,23 +4221,23 @@
         <v>65</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F68" s="1"/>
       <c r="G68" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="69" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -4229,23 +4245,23 @@
         <v>66</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C69" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="D69" s="1" t="s">
         <v>417</v>
       </c>
-      <c r="D69" s="1" t="s">
-        <v>418</v>
-      </c>
       <c r="E69" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F69" s="1"/>
       <c r="G69" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="70" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -4253,13 +4269,13 @@
         <v>67</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>128</v>
@@ -4277,19 +4293,19 @@
         <v>68</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C71" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="D71" s="1" t="s">
+      <c r="E71" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="E71" s="1" t="s">
-        <v>409</v>
-      </c>
       <c r="F71" s="1" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="G71" s="2" t="s">
         <v>19</v>
@@ -4301,19 +4317,19 @@
         <v>69</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C72" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="F72" s="1" t="s">
         <v>410</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>413</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>412</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>411</v>
       </c>
       <c r="G72" s="2" t="s">
         <v>19</v>
@@ -4325,23 +4341,23 @@
         <v>70</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C73" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="D73" s="1" t="s">
+      <c r="E73" s="1" t="s">
         <v>421</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>422</v>
       </c>
       <c r="F73" s="1"/>
       <c r="G73" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H73" s="3" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="74" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -4349,23 +4365,23 @@
         <v>71</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="D74" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="E74" s="1" t="s">
         <v>426</v>
-      </c>
-      <c r="E74" s="1" t="s">
-        <v>427</v>
       </c>
       <c r="F74" s="1"/>
       <c r="G74" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H74" s="3" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="75" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -4373,23 +4389,23 @@
         <v>72</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="F75" s="1"/>
       <c r="G75" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H75" s="3" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="76" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -4397,13 +4413,13 @@
         <v>73</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C76" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="D76" s="1" t="s">
         <v>430</v>
-      </c>
-      <c r="D76" s="1" t="s">
-        <v>431</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>128</v>
@@ -4421,19 +4437,19 @@
         <v>74</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C77" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="D77" s="1" t="s">
         <v>435</v>
       </c>
-      <c r="D77" s="1" t="s">
+      <c r="E77" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="E77" s="1" t="s">
-        <v>437</v>
-      </c>
       <c r="F77" s="1" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="G77" s="2" t="s">
         <v>19</v>
@@ -4445,13 +4461,13 @@
         <v>75</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C78" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D78" s="1" t="s">
         <v>438</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>439</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>128</v>
@@ -4469,23 +4485,23 @@
         <v>76</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C79" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="D79" s="1" t="s">
         <v>440</v>
       </c>
-      <c r="D79" s="1" t="s">
-        <v>441</v>
-      </c>
       <c r="E79" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F79" s="1"/>
       <c r="G79" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H79" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="80" spans="1:8" s="6" customFormat="1" ht="105" x14ac:dyDescent="0.25">
@@ -4493,23 +4509,23 @@
         <v>77</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D80" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="E80" s="1" t="s">
         <v>395</v>
-      </c>
-      <c r="E80" s="1" t="s">
-        <v>396</v>
       </c>
       <c r="F80" s="1"/>
       <c r="G80" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H80" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="81" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -4517,23 +4533,23 @@
         <v>78</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="F81" s="1"/>
       <c r="G81" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H81" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="82" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -4541,13 +4557,13 @@
         <v>79</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="E82" s="1" t="s">
         <v>128</v>
@@ -4565,19 +4581,19 @@
         <v>80</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="G83" s="2" t="s">
         <v>19</v>
@@ -4589,13 +4605,13 @@
         <v>81</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E84" s="1" t="s">
         <v>128</v>
@@ -4613,19 +4629,19 @@
         <v>82</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>19</v>
@@ -4637,13 +4653,13 @@
         <v>83</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E86" s="1" t="s">
         <v>128</v>
@@ -4661,19 +4677,19 @@
         <v>84</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D87" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="E87" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="E87" s="1" t="s">
-        <v>288</v>
-      </c>
       <c r="F87" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>19</v>
@@ -4685,19 +4701,19 @@
         <v>85</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C88" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="D88" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="D88" s="1" t="s">
+      <c r="E88" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="E88" s="1" t="s">
-        <v>404</v>
-      </c>
       <c r="F88" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="G88" s="2" t="s">
         <v>19</v>
@@ -4709,25 +4725,25 @@
         <v>86</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C89" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="D89" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="D89" s="1" t="s">
-        <v>346</v>
-      </c>
       <c r="E89" s="1" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G89" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="90" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -4735,23 +4751,23 @@
         <v>87</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="F90" s="1"/>
       <c r="G90" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H90" s="3" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="91" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -4759,23 +4775,23 @@
         <v>88</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="F91" s="1"/>
       <c r="G91" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H91" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="92" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -4783,13 +4799,13 @@
         <v>89</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="E92" s="1" t="s">
         <v>128</v>
@@ -4807,23 +4823,23 @@
         <v>90</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="F93" s="1"/>
       <c r="G93" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="94" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -4831,13 +4847,13 @@
         <v>91</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E94" s="1" t="s">
         <v>128</v>
@@ -4855,19 +4871,19 @@
         <v>92</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="G95" s="2" t="s">
         <v>19</v>
@@ -4879,13 +4895,13 @@
         <v>93</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E96" s="1" t="s">
         <v>128</v>
@@ -4903,23 +4919,23 @@
         <v>94</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D97" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="E97" s="1" t="s">
         <v>287</v>
-      </c>
-      <c r="E97" s="1" t="s">
-        <v>288</v>
       </c>
       <c r="F97" s="1"/>
       <c r="G97" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H97" s="3" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="98" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -4927,23 +4943,23 @@
         <v>95</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="D98" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="E98" s="1" t="s">
         <v>369</v>
-      </c>
-      <c r="E98" s="1" t="s">
-        <v>370</v>
       </c>
       <c r="F98" s="1"/>
       <c r="G98" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="99" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -4951,23 +4967,23 @@
         <v>96</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F99" s="1"/>
       <c r="G99" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H99" s="3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="100" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -4975,23 +4991,23 @@
         <v>97</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="F100" s="1"/>
       <c r="G100" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="101" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -4999,25 +5015,25 @@
         <v>98</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="C101" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="D101" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="D101" s="1" t="s">
+      <c r="E101" s="1" t="s">
         <v>316</v>
       </c>
-      <c r="E101" s="1" t="s">
-        <v>317</v>
-      </c>
       <c r="F101" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="G101" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H101" s="3" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="102" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -5025,16 +5041,16 @@
         <v>99</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F102" s="1"/>
       <c r="G102" s="2" t="s">
@@ -5047,23 +5063,23 @@
         <v>100</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F103" s="1"/>
       <c r="G103" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="104" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -5071,13 +5087,13 @@
         <v>101</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E104" s="1" t="s">
         <v>128</v>
@@ -5095,25 +5111,25 @@
         <v>102</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G105" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H105" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="106" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -5121,13 +5137,13 @@
         <v>103</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E106" s="1" t="s">
         <v>128</v>
@@ -5145,25 +5161,25 @@
         <v>104</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G107" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H107" s="3" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="108" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -5171,13 +5187,13 @@
         <v>105</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E108" s="1" t="s">
         <v>128</v>
@@ -5195,19 +5211,19 @@
         <v>106</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="D109" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="E109" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="E109" s="1" t="s">
-        <v>288</v>
-      </c>
       <c r="F109" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G109" s="2" t="s">
         <v>19</v>
@@ -5219,25 +5235,25 @@
         <v>107</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C110" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="D110" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="D110" s="1" t="s">
+      <c r="E110" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="E110" s="1" t="s">
-        <v>295</v>
-      </c>
       <c r="F110" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G110" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H110" s="3" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="111" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -5245,19 +5261,19 @@
         <v>108</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G111" s="2" t="s">
         <v>19</v>
@@ -5269,16 +5285,16 @@
         <v>109</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F112" s="1"/>
       <c r="G112" s="2" t="s">
@@ -5291,13 +5307,13 @@
         <v>110</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="E113" s="1" t="s">
         <v>128</v>
@@ -5315,19 +5331,19 @@
         <v>111</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F114" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G114" s="2" t="s">
         <v>19</v>
@@ -5339,13 +5355,13 @@
         <v>112</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E115" s="1" t="s">
         <v>128</v>
@@ -5363,19 +5379,19 @@
         <v>113</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="F116" s="1" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="G116" s="2" t="s">
         <v>19</v>
@@ -5387,13 +5403,13 @@
         <v>114</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E117" s="1" t="s">
         <v>128</v>
@@ -5413,25 +5429,25 @@
         <v>115</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D118" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="E118" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="E118" s="1" t="s">
-        <v>288</v>
-      </c>
       <c r="F118" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G118" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H118" s="3" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="119" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -5439,23 +5455,23 @@
         <v>116</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C119" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="D119" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="D119" s="1" t="s">
+      <c r="E119" s="1" t="s">
         <v>306</v>
-      </c>
-      <c r="E119" s="1" t="s">
-        <v>307</v>
       </c>
       <c r="F119" s="1"/>
       <c r="G119" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H119" s="3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="120" spans="1:8" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -5463,23 +5479,23 @@
         <v>117</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F120" s="1"/>
       <c r="G120" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H120" s="3" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="121" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -5487,23 +5503,23 @@
         <v>118</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F121" s="1"/>
       <c r="G121" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H121" s="3" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="122" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -5511,25 +5527,25 @@
         <v>119</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D122" s="1" t="s">
         <v>140</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F122" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G122" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H122" s="3" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="123" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -5537,19 +5553,19 @@
         <v>120</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E123" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F123" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G123" s="2" t="s">
         <v>19</v>
@@ -5561,25 +5577,25 @@
         <v>121</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E124" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F124" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G124" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H124" s="3" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="125" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -5587,13 +5603,13 @@
         <v>122</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="E125" s="1" t="s">
         <v>128</v>
@@ -5611,25 +5627,25 @@
         <v>123</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="E126" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F126" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G126" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H126" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="127" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -5637,13 +5653,13 @@
         <v>124</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E127" s="1" t="s">
         <v>128</v>
@@ -5661,19 +5677,19 @@
         <v>125</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F128" s="1" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="G128" s="2" t="s">
         <v>19</v>
@@ -5685,13 +5701,13 @@
         <v>126</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E129" s="1" t="s">
         <v>128</v>
@@ -5709,19 +5725,19 @@
         <v>127</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D130" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="E130" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="E130" s="1" t="s">
-        <v>288</v>
-      </c>
       <c r="F130" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="G130" s="2" t="s">
         <v>19</v>
@@ -5733,23 +5749,23 @@
         <v>128</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D131" s="1" t="s">
         <v>141</v>
       </c>
       <c r="E131" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F131" s="1"/>
       <c r="G131" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H131" s="3" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="132" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -5757,23 +5773,23 @@
         <v>129</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D132" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="E132" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="E132" s="1" t="s">
-        <v>248</v>
       </c>
       <c r="F132" s="1"/>
       <c r="G132" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H132" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="133" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -5781,23 +5797,23 @@
         <v>130</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D133" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="E133" s="1" t="s">
         <v>250</v>
-      </c>
-      <c r="E133" s="1" t="s">
-        <v>251</v>
       </c>
       <c r="F133" s="1"/>
       <c r="G133" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H133" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="134" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -5805,23 +5821,23 @@
         <v>131</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D134" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="E134" s="1" t="s">
         <v>255</v>
-      </c>
-      <c r="E134" s="1" t="s">
-        <v>256</v>
       </c>
       <c r="F134" s="1"/>
       <c r="G134" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H134" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="135" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -5829,23 +5845,23 @@
         <v>132</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="C135" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D135" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="E135" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="D135" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="E135" s="1" t="s">
-        <v>258</v>
       </c>
       <c r="F135" s="1"/>
       <c r="G135" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="136" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -5853,23 +5869,23 @@
         <v>133</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="C136" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D136" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="D136" s="1" t="s">
+      <c r="E136" s="1" t="s">
         <v>260</v>
-      </c>
-      <c r="E136" s="1" t="s">
-        <v>261</v>
       </c>
       <c r="F136" s="1"/>
       <c r="G136" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H136" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="137" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -5877,23 +5893,23 @@
         <v>134</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="C137" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="D137" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="D137" s="1" t="s">
+      <c r="E137" s="1" t="s">
         <v>263</v>
-      </c>
-      <c r="E137" s="1" t="s">
-        <v>264</v>
       </c>
       <c r="F137" s="1"/>
       <c r="G137" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H137" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="138" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -5901,23 +5917,23 @@
         <v>135</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="C138" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="D138" s="1" t="s">
         <v>244</v>
       </c>
-      <c r="D138" s="1" t="s">
+      <c r="E138" s="1" t="s">
         <v>245</v>
-      </c>
-      <c r="E138" s="1" t="s">
-        <v>246</v>
       </c>
       <c r="F138" s="1"/>
       <c r="G138" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H138" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="139" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -5925,23 +5941,23 @@
         <v>136</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="C139" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D139" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="D139" s="1" t="s">
+      <c r="E139" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="E139" s="1" t="s">
-        <v>268</v>
       </c>
       <c r="F139" s="1"/>
       <c r="G139" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H139" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="140" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -5949,25 +5965,25 @@
         <v>137</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D140" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="E140" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="F140" s="1" t="s">
         <v>269</v>
-      </c>
-      <c r="E140" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="F140" s="1" t="s">
-        <v>270</v>
       </c>
       <c r="G140" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H140" s="3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="141" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -5975,25 +5991,25 @@
         <v>138</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C141" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="D141" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="D141" s="1" t="s">
+      <c r="E141" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="E141" s="1" t="s">
-        <v>234</v>
-      </c>
       <c r="F141" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G141" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H141" s="3" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="142" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -6001,23 +6017,23 @@
         <v>139</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D142" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="E142" s="1" t="s">
         <v>235</v>
-      </c>
-      <c r="E142" s="1" t="s">
-        <v>236</v>
       </c>
       <c r="F142" s="1"/>
       <c r="G142" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H142" s="3" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="143" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -6025,13 +6041,13 @@
         <v>140</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D143" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E143" s="1" t="s">
         <v>128</v>
@@ -6049,13 +6065,13 @@
         <v>141</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D144" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E144" s="1" t="s">
         <v>128</v>
@@ -6067,7 +6083,7 @@
         <v>20</v>
       </c>
       <c r="H144" s="3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="145" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -6075,7 +6091,7 @@
         <v>142</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>100</v>
@@ -6084,10 +6100,10 @@
         <v>142</v>
       </c>
       <c r="E145" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F145" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G145" s="2" t="s">
         <v>19</v>
@@ -6099,23 +6115,23 @@
         <v>143</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D146" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="E146" s="1" t="s">
         <v>229</v>
-      </c>
-      <c r="E146" s="1" t="s">
-        <v>230</v>
       </c>
       <c r="F146" s="1"/>
       <c r="G146" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H146" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="147" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -6123,25 +6139,25 @@
         <v>144</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D147" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="E147" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="E147" s="1" t="s">
+      <c r="F147" s="1" t="s">
         <v>223</v>
-      </c>
-      <c r="F147" s="1" t="s">
-        <v>224</v>
       </c>
       <c r="G147" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H147" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="148" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -6149,19 +6165,19 @@
         <v>145</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D148" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="E148" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="E148" s="1" t="s">
-        <v>227</v>
-      </c>
       <c r="F148" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="G148" s="2" t="s">
         <v>19</v>
@@ -6173,13 +6189,13 @@
         <v>146</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D149" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E149" s="1"/>
       <c r="F149" s="1"/>
@@ -6187,7 +6203,7 @@
         <v>20</v>
       </c>
       <c r="H149" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="150" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -6195,23 +6211,23 @@
         <v>147</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D150" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="E150" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="E150" s="1" t="s">
-        <v>211</v>
       </c>
       <c r="F150" s="1"/>
       <c r="G150" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H150" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="151" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -6219,23 +6235,23 @@
         <v>148</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D151" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E151" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F151" s="1"/>
       <c r="G151" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H151" s="3" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="152" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -6243,23 +6259,23 @@
         <v>149</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="C152" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D152" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="D152" s="1" t="s">
+      <c r="E152" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="E152" s="1" t="s">
-        <v>217</v>
       </c>
       <c r="F152" s="1"/>
       <c r="G152" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H152" s="3" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="153" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -6267,23 +6283,23 @@
         <v>150</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D153" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="E153" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="E153" s="1" t="s">
-        <v>209</v>
       </c>
       <c r="F153" s="1"/>
       <c r="G153" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H153" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="154" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -6291,16 +6307,16 @@
         <v>151</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D154" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E154" s="1" t="s">
         <v>195</v>
-      </c>
-      <c r="E154" s="1" t="s">
-        <v>196</v>
       </c>
       <c r="F154" s="1"/>
       <c r="G154" s="2" t="s">
@@ -6313,19 +6329,19 @@
         <v>152</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E155" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F155" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G155" s="2" t="s">
         <v>19</v>
@@ -6337,19 +6353,19 @@
         <v>153</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E156" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F156" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G156" s="2" t="s">
         <v>19</v>
@@ -6361,19 +6377,19 @@
         <v>154</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C157" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="D157" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="D157" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="E157" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F157" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="G157" s="2" t="s">
         <v>19</v>
@@ -6385,23 +6401,23 @@
         <v>155</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D158" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E158" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="E158" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="F158" s="1"/>
       <c r="G158" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H158" s="3" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="159" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -6409,23 +6425,23 @@
         <v>156</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D159" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E159" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F159" s="1"/>
       <c r="G159" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H159" s="3" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="160" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -6433,13 +6449,13 @@
         <v>157</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E160" s="1" t="s">
         <v>128</v>
@@ -6455,7 +6471,7 @@
         <v>158</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>101</v>
@@ -6464,10 +6480,10 @@
         <v>143</v>
       </c>
       <c r="E161" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F161" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G161" s="2" t="s">
         <v>19</v>
@@ -6479,23 +6495,23 @@
         <v>159</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C162" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="D162" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D162" s="1" t="s">
+      <c r="E162" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="E162" s="1" t="s">
-        <v>179</v>
       </c>
       <c r="F162" s="1"/>
       <c r="G162" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H162" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="163" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -6503,7 +6519,7 @@
         <v>160</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>102</v>
@@ -6512,14 +6528,14 @@
         <v>144</v>
       </c>
       <c r="E163" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F163" s="1"/>
       <c r="G163" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H163" s="3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="164" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -6527,23 +6543,23 @@
         <v>161</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="C164" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D164" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="D164" s="1" t="s">
+      <c r="E164" s="1" t="s">
         <v>172</v>
-      </c>
-      <c r="E164" s="1" t="s">
-        <v>173</v>
       </c>
       <c r="F164" s="1"/>
       <c r="G164" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H164" s="3" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="165" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -6551,7 +6567,7 @@
         <v>162</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>53</v>
@@ -6577,7 +6593,7 @@
         <v>163</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>58</v>
@@ -6593,7 +6609,7 @@
         <v>8</v>
       </c>
       <c r="H166" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="167" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -6601,7 +6617,7 @@
         <v>164</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>61</v>

</xml_diff>

<commit_message>
Actualizados testscases web and app
</commit_message>
<xml_diff>
--- a/App/TestCases_App/User_admin.xlsx
+++ b/App/TestCases_App/User_admin.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nerea QA\PycharmProjects\KOVAI\App\TestCases_App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D61B70F6-F3B1-422D-9F63-1706AE21C0D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74648248-8637-41C9-A243-79082D307A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1888,9 +1888,6 @@
     <t>1. The search is displayed</t>
   </si>
   <si>
-    <t>1.The user writes a world in the box of the search</t>
-  </si>
-  <si>
     <t>Menus_types: search</t>
   </si>
   <si>
@@ -2006,9 +2003,6 @@
     <t>1. The user sees the menu_type</t>
   </si>
   <si>
-    <t>Se edita la carta, no se ve solo</t>
-  </si>
-  <si>
     <t>1.The user clicks eye icon (carta personalizada)
 2. Clicks "Cancelar"</t>
   </si>
@@ -2203,11 +2197,6 @@
     <t>1. Select numbers of people
 2. Select several products
 3. Add fee</t>
-  </si>
-  <si>
-    <t>1. Select numbers of people
-2. Select several products with his modifiers
-3. Select menu</t>
   </si>
   <si>
     <t>1. Select numbers of people, clicks "Aceptar"
@@ -2283,12 +2272,6 @@
     <t>1. The product is added.</t>
   </si>
   <si>
-    <t>No veo variación al cambiar de menú</t>
-  </si>
-  <si>
-    <t>1. The products shown are the menu's product.</t>
-  </si>
-  <si>
     <t>The fee is added</t>
   </si>
   <si>
@@ -2328,6 +2311,25 @@
   <si>
     <t>No hay tickets
 15/05/26: El ticket practicamente no se ve, y ademas dice que el pago total de 13,80e está hecho con tarjeta, cuando parte esta hecho con tarjeta y parte con efectivo: HISTIC001.jpg</t>
+  </si>
+  <si>
+    <t>1. The user writes a world in the box of the search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se edita la carta, no se ve solo
+</t>
+  </si>
+  <si>
+    <t>No veo variación al cambiar de menú
+18/05/26: El menú desplegable, donde escoges "CARTA", se ha quedado vacio sin carta: MEN007.jpg</t>
+  </si>
+  <si>
+    <t>1. The menu is selected.</t>
+  </si>
+  <si>
+    <t>1. Select numbers of people
+2. Select several products with his modifiers
+3. Select menu (button "CARTA")</t>
   </si>
 </sst>
 </file>
@@ -2884,13 +2886,13 @@
         <v>30</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>674</v>
+        <v>669</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>673</v>
+        <v>668</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="2" t="s">
@@ -2914,7 +2916,7 @@
         <v>9</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>672</v>
+        <v>667</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="2" t="s">
@@ -2932,13 +2934,13 @@
         <v>32</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>663</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>657</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>666</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>659</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>671</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="2" t="s">
@@ -2959,17 +2961,17 @@
         <v>565</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>660</v>
+        <v>681</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>670</v>
+        <v>680</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>669</v>
+        <v>679</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -2980,16 +2982,16 @@
         <v>34</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>13</v>
@@ -3004,10 +3006,10 @@
         <v>35</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>21</v>
@@ -3028,20 +3030,20 @@
         <v>36</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
     </row>
     <row r="11" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -3052,16 +3054,16 @@
         <v>37</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>13</v>
@@ -3079,7 +3081,7 @@
         <v>559</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>21</v>
@@ -3103,7 +3105,7 @@
         <v>564</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>23</v>
@@ -3127,7 +3129,7 @@
         <v>560</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
@@ -3438,10 +3440,10 @@
         <v>77</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>575</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>576</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>571</v>
@@ -3471,7 +3473,7 @@
         <v>8</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>681</v>
+        <v>676</v>
       </c>
     </row>
     <row r="29" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -3524,17 +3526,17 @@
         <v>129</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
     </row>
     <row r="32" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -3556,7 +3558,7 @@
         <v>8</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="33" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3576,7 +3578,7 @@
         <v>8</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="34" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -3593,14 +3595,14 @@
         <v>144</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="35" spans="1:8" s="6" customFormat="1" ht="60" x14ac:dyDescent="0.25">
@@ -3758,7 +3760,7 @@
         <v>8</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="42" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3769,7 +3771,7 @@
         <v>450</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>156</v>
@@ -3780,7 +3782,7 @@
         <v>8</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="43" spans="1:8" s="6" customFormat="1" ht="105" x14ac:dyDescent="0.25">
@@ -3791,20 +3793,20 @@
         <v>451</v>
       </c>
       <c r="C43" s="1" t="s">
+        <v>632</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>633</v>
+      </c>
+      <c r="E43" s="1" t="s">
         <v>634</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>635</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>636</v>
       </c>
       <c r="F43" s="1"/>
       <c r="G43" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
     </row>
     <row r="44" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -3815,10 +3817,10 @@
         <v>452</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>120</v>
@@ -3839,10 +3841,10 @@
         <v>453</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="E45" s="1"/>
       <c r="F45" s="1"/>
@@ -3850,7 +3852,7 @@
         <v>8</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="46" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -3861,10 +3863,10 @@
         <v>103</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="E46" s="1"/>
       <c r="F46" s="1"/>
@@ -3872,7 +3874,7 @@
         <v>8</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="47" spans="1:8" s="6" customFormat="1" x14ac:dyDescent="0.25">
@@ -3891,7 +3893,7 @@
       <c r="E47" s="1"/>
       <c r="F47" s="1"/>
       <c r="G47" s="2" t="s">
-        <v>680</v>
+        <v>675</v>
       </c>
       <c r="H47" s="7" t="s">
         <v>447</v>
@@ -3908,13 +3910,13 @@
         <v>443</v>
       </c>
       <c r="D48" s="1" t="s">
+        <v>598</v>
+      </c>
+      <c r="E48" s="1" t="s">
         <v>599</v>
       </c>
-      <c r="E48" s="1" t="s">
-        <v>600</v>
-      </c>
       <c r="F48" s="1" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G48" s="2" t="s">
         <v>13</v>
@@ -3932,13 +3934,13 @@
         <v>444</v>
       </c>
       <c r="D49" s="1" t="s">
+        <v>600</v>
+      </c>
+      <c r="E49" s="1" t="s">
         <v>601</v>
       </c>
-      <c r="E49" s="1" t="s">
-        <v>602</v>
-      </c>
       <c r="F49" s="1" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="G49" s="2" t="s">
         <v>13</v>
@@ -3953,13 +3955,13 @@
         <v>107</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="F50" s="1"/>
       <c r="G50" s="2" t="s">
@@ -3977,10 +3979,10 @@
         <v>108</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>120</v>
@@ -4000,20 +4002,20 @@
         <v>109</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="D52" s="1" t="s">
+        <v>603</v>
+      </c>
+      <c r="E52" s="1" t="s">
         <v>604</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>605</v>
       </c>
       <c r="F52" s="1"/>
       <c r="G52" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H52" s="3" t="s">
-        <v>606</v>
+        <v>678</v>
       </c>
     </row>
     <row r="53" spans="1:8" s="6" customFormat="1" ht="45" x14ac:dyDescent="0.25">
@@ -4024,10 +4026,10 @@
         <v>110</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>120</v>
@@ -4046,13 +4048,13 @@
         <v>454</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="F54" s="1"/>
       <c r="G54" s="2" t="s">
@@ -4070,20 +4072,20 @@
         <v>111</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="F55" s="1"/>
       <c r="G55" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
     </row>
     <row r="56" spans="1:8" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -4094,20 +4096,20 @@
         <v>112</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="F56" s="1"/>
       <c r="G56" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>675</v>
+        <v>670</v>
       </c>
     </row>
     <row r="57" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -4118,10 +4120,10 @@
         <v>455</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>120</v>
@@ -4142,20 +4144,20 @@
         <v>455</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>676</v>
+        <v>671</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>678</v>
+        <v>673</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>679</v>
+        <v>674</v>
       </c>
       <c r="F58" s="1"/>
       <c r="G58" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>677</v>
+        <v>672</v>
       </c>
     </row>
     <row r="59" spans="1:8" s="6" customFormat="1" ht="75" x14ac:dyDescent="0.25">
@@ -4166,20 +4168,20 @@
         <v>113</v>
       </c>
       <c r="C59" s="1" t="s">
+        <v>611</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>622</v>
+      </c>
+      <c r="E59" s="1" t="s">
         <v>613</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>624</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>615</v>
       </c>
       <c r="F59" s="1"/>
       <c r="G59" s="2" t="s">
         <v>8</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
     </row>
     <row r="60" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -4190,10 +4192,10 @@
         <v>114</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>120</v>
@@ -4214,16 +4216,16 @@
         <v>115</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>13</v>
@@ -4238,10 +4240,10 @@
         <v>116</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>120</v>
@@ -4262,16 +4264,16 @@
         <v>117</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>572</v>
+        <v>677</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>13</v>
@@ -4308,13 +4310,13 @@
         <v>434</v>
       </c>
       <c r="D65" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="E65" s="1" t="s">
         <v>591</v>
       </c>
-      <c r="E65" s="1" t="s">
-        <v>592</v>
-      </c>
       <c r="F65" s="1" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="G65" s="2" t="s">
         <v>13</v>
@@ -4332,7 +4334,7 @@
         <v>440</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>120</v>
@@ -4356,13 +4358,13 @@
         <v>436</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>13</v>
@@ -4404,13 +4406,13 @@
         <v>437</v>
       </c>
       <c r="D69" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="E69" s="1" t="s">
         <v>597</v>
       </c>
-      <c r="E69" s="1" t="s">
-        <v>598</v>
-      </c>
       <c r="F69" s="1" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="G69" s="2" t="s">
         <v>13</v>
@@ -4428,7 +4430,7 @@
         <v>442</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>120</v>
@@ -4500,7 +4502,7 @@
         <v>405</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>120</v>
@@ -5404,7 +5406,7 @@
         <v>8</v>
       </c>
       <c r="H110" s="3" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="111" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -6696,7 +6698,7 @@
         <v>162</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>93</v>
@@ -6720,7 +6722,7 @@
         <v>163</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>168</v>
@@ -6744,7 +6746,7 @@
         <v>164</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>94</v>
@@ -6768,7 +6770,7 @@
         <v>165</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>162</v>
@@ -6784,7 +6786,7 @@
         <v>8</v>
       </c>
       <c r="H167" s="3" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
     </row>
     <row r="168" spans="1:8" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -6792,7 +6794,7 @@
         <v>166</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>45</v>
@@ -6818,7 +6820,7 @@
         <v>167</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="C169" s="1" t="s">
         <v>50</v>
@@ -6842,7 +6844,7 @@
         <v>168</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>665</v>
+        <v>662</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>53</v>

</xml_diff>